<commit_message>
chỉnh sửa phần xử lí drop cho missing, phần isolation forest để chạy hiệu quả hơn.
</commit_message>
<xml_diff>
--- a/outputs/results/experiment_results.xlsx
+++ b/outputs/results/experiment_results.xlsx
@@ -485,16 +485,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7279407279681209</v>
+        <v>0.7210339436317338</v>
       </c>
       <c r="E2" t="n">
-        <v>8.7294274070847</v>
+        <v>8.579833232622121</v>
       </c>
       <c r="F2" t="n">
-        <v>1.488941607420576</v>
+        <v>1.496604910981668</v>
       </c>
       <c r="G2" t="n">
-        <v>2.920838841138348</v>
+        <v>2.898606411703435</v>
       </c>
     </row>
     <row r="3">
@@ -514,16 +514,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.6893743936746362</v>
+        <v>0.7510702611565285</v>
       </c>
       <c r="E3" t="n">
-        <v>9.966885748636415</v>
+        <v>7.656041289473947</v>
       </c>
       <c r="F3" t="n">
-        <v>1.57589644650905</v>
+        <v>1.464502076096448</v>
       </c>
       <c r="G3" t="n">
-        <v>3.13131259038262</v>
+        <v>2.718897244795108</v>
       </c>
     </row>
     <row r="4">
@@ -543,16 +543,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.7597737896642778</v>
+        <v>0.7541928888739091</v>
       </c>
       <c r="E4" t="n">
-        <v>7.70801615671096</v>
+        <v>7.56000227522441</v>
       </c>
       <c r="F4" t="n">
-        <v>1.484660811812581</v>
+        <v>1.474694267909985</v>
       </c>
       <c r="G4" t="n">
-        <v>2.705476920323415</v>
+        <v>2.682392262736036</v>
       </c>
     </row>
     <row r="5">
@@ -572,16 +572,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7384313989539995</v>
+        <v>0.7314217202433815</v>
       </c>
       <c r="E5" t="n">
-        <v>8.392818586003585</v>
+        <v>8.260348517721848</v>
       </c>
       <c r="F5" t="n">
-        <v>1.455022630045817</v>
+        <v>1.464084904706317</v>
       </c>
       <c r="G5" t="n">
-        <v>2.874622307341991</v>
+        <v>2.854148826320528</v>
       </c>
     </row>
     <row r="6">
@@ -601,16 +601,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6973501461986943</v>
+        <v>0.7591824763890805</v>
       </c>
       <c r="E6" t="n">
-        <v>9.710971836364093</v>
+        <v>7.406543358619767</v>
       </c>
       <c r="F6" t="n">
-        <v>1.547033802742398</v>
+        <v>1.440416400603951</v>
       </c>
       <c r="G6" t="n">
-        <v>3.097020781186702</v>
+        <v>2.684299947141111</v>
       </c>
     </row>
     <row r="7">
@@ -630,16 +630,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7684014337337335</v>
+        <v>0.7625833435452005</v>
       </c>
       <c r="E7" t="n">
-        <v>7.431185332177795</v>
+        <v>7.301946858867508</v>
       </c>
       <c r="F7" t="n">
-        <v>1.461107580309341</v>
+        <v>1.453374252935564</v>
       </c>
       <c r="G7" t="n">
-        <v>2.668931832342693</v>
+        <v>2.647721551907941</v>
       </c>
     </row>
     <row r="8">
@@ -688,16 +688,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.688369542223954</v>
+        <v>0.7404458018019563</v>
       </c>
       <c r="E9" t="n">
-        <v>9.584454082809753</v>
+        <v>7.982805379111669</v>
       </c>
       <c r="F9" t="n">
-        <v>1.523528669025294</v>
+        <v>1.474224465462455</v>
       </c>
       <c r="G9" t="n">
-        <v>3.068408159475235</v>
+        <v>2.769164926398047</v>
       </c>
     </row>
     <row r="10">
@@ -775,16 +775,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6937095556455837</v>
+        <v>0.7484151104614505</v>
       </c>
       <c r="E12" t="n">
-        <v>9.420217525810633</v>
+        <v>7.737702658845629</v>
       </c>
       <c r="F12" t="n">
-        <v>1.501678063253718</v>
+        <v>1.450233806848774</v>
       </c>
       <c r="G12" t="n">
-        <v>3.048321474812925</v>
+        <v>2.73523744632631</v>
       </c>
     </row>
     <row r="13">
@@ -862,16 +862,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.6903983233378498</v>
+        <v>0.74168487282217</v>
       </c>
       <c r="E15" t="n">
-        <v>9.522057231202329</v>
+        <v>7.944696718670292</v>
       </c>
       <c r="F15" t="n">
-        <v>1.528527446624669</v>
+        <v>1.451467819982617</v>
       </c>
       <c r="G15" t="n">
-        <v>3.057944844552671</v>
+        <v>2.756385478425933</v>
       </c>
     </row>
     <row r="16">
@@ -949,16 +949,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.6984895474710907</v>
+        <v>0.7498136265114418</v>
       </c>
       <c r="E18" t="n">
-        <v>9.273204899077268</v>
+        <v>7.694690133815593</v>
       </c>
       <c r="F18" t="n">
-        <v>1.499214670416661</v>
+        <v>1.429013677817497</v>
       </c>
       <c r="G18" t="n">
-        <v>3.023727105358379</v>
+        <v>2.721600451197589</v>
       </c>
     </row>
     <row r="19">
@@ -1036,16 +1036,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.6896906156082456</v>
+        <v>0.7520867366290632</v>
       </c>
       <c r="E21" t="n">
-        <v>9.543823371414835</v>
+        <v>7.624778740356194</v>
       </c>
       <c r="F21" t="n">
-        <v>1.526324702240442</v>
+        <v>1.455935263582135</v>
       </c>
       <c r="G21" t="n">
-        <v>3.062139175540382</v>
+        <v>2.703583174802635</v>
       </c>
     </row>
     <row r="22">
@@ -1123,16 +1123,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.6968320813903595</v>
+        <v>0.759473054982568</v>
       </c>
       <c r="E24" t="n">
-        <v>9.324181647813425</v>
+        <v>7.397606372143528</v>
       </c>
       <c r="F24" t="n">
-        <v>1.502992490705599</v>
+        <v>1.433710724260695</v>
       </c>
       <c r="G24" t="n">
-        <v>3.032739646614405</v>
+        <v>2.673831396952504</v>
       </c>
     </row>
     <row r="25">
@@ -1242,16 +1242,16 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.792234478173077</v>
+        <v>0.7866208433183421</v>
       </c>
       <c r="F2" t="n">
-        <v>6.666466564207651</v>
+        <v>6.562653548177084</v>
       </c>
       <c r="G2" t="n">
-        <v>1.15957650273224</v>
+        <v>1.1729296875</v>
       </c>
       <c r="H2" t="n">
-        <v>2.58195014750627</v>
+        <v>2.56176766085004</v>
       </c>
     </row>
     <row r="3">
@@ -1272,20 +1272,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.7607017181311997</v>
+        <v>0.8336727685103763</v>
       </c>
       <c r="F3" t="n">
-        <v>7.678242188228045</v>
+        <v>5.115532430013021</v>
       </c>
       <c r="G3" t="n">
-        <v>1.28388548304942</v>
+        <v>1.10529296875</v>
       </c>
       <c r="H3" t="n">
-        <v>2.770964126117125</v>
+        <v>2.261754281528615</v>
       </c>
     </row>
     <row r="4">
@@ -1310,16 +1310,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.8714480623028008</v>
+        <v>0.8664022178760558</v>
       </c>
       <c r="F4" t="n">
-        <v>4.124780603089613</v>
+        <v>4.108910975744135</v>
       </c>
       <c r="G4" t="n">
-        <v>1.081322766388076</v>
+        <v>1.081957858672392</v>
       </c>
       <c r="H4" t="n">
-        <v>2.030955588655157</v>
+        <v>2.027044887451715</v>
       </c>
     </row>
     <row r="5">
@@ -1344,16 +1344,16 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.7895576072989532</v>
+        <v>0.7838902467226974</v>
       </c>
       <c r="F5" t="n">
-        <v>6.752357957650273</v>
+        <v>6.646635319010417</v>
       </c>
       <c r="G5" t="n">
-        <v>1.163811475409836</v>
+        <v>1.177513020833333</v>
       </c>
       <c r="H5" t="n">
-        <v>2.598529960891402</v>
+        <v>2.578106925441693</v>
       </c>
     </row>
     <row r="6">
@@ -1374,20 +1374,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.7606033590963361</v>
+        <v>0.8332430227830193</v>
       </c>
       <c r="F6" t="n">
-        <v>7.681398184523484</v>
+        <v>5.12874961751302</v>
       </c>
       <c r="G6" t="n">
-        <v>1.286100831315334</v>
+        <v>1.104407552083333</v>
       </c>
       <c r="H6" t="n">
-        <v>2.771533543820728</v>
+        <v>2.264674285082299</v>
       </c>
     </row>
     <row r="7">
@@ -1412,16 +1412,16 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.8714480623028008</v>
+        <v>0.8664022178760558</v>
       </c>
       <c r="F7" t="n">
-        <v>4.124780603089613</v>
+        <v>4.108910975744135</v>
       </c>
       <c r="G7" t="n">
-        <v>1.081322766388076</v>
+        <v>1.081957858672392</v>
       </c>
       <c r="H7" t="n">
-        <v>2.030955588655157</v>
+        <v>2.027044887451715</v>
       </c>
     </row>
     <row r="8">
@@ -1476,20 +1476,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.7633867899815057</v>
+        <v>0.8352912414456735</v>
       </c>
       <c r="F9" t="n">
-        <v>7.277236195052044</v>
+        <v>5.065754947916666</v>
       </c>
       <c r="G9" t="n">
-        <v>1.226473334554635</v>
+        <v>1.091197916666667</v>
       </c>
       <c r="H9" t="n">
-        <v>2.697635296894679</v>
+        <v>2.250723205531206</v>
       </c>
     </row>
     <row r="10">
@@ -1578,20 +1578,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.7633681944944954</v>
+        <v>0.8344501638320561</v>
       </c>
       <c r="F12" t="n">
-        <v>7.277808114731106</v>
+        <v>5.091622989908855</v>
       </c>
       <c r="G12" t="n">
-        <v>1.227003489121217</v>
+        <v>1.09474609375</v>
       </c>
       <c r="H12" t="n">
-        <v>2.697741298703622</v>
+        <v>2.256462494682518</v>
       </c>
     </row>
     <row r="13">
@@ -1680,20 +1680,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.7665019904937718</v>
+        <v>0.8370011472178656</v>
       </c>
       <c r="F15" t="n">
-        <v>7.181425610677084</v>
+        <v>5.013165372826788</v>
       </c>
       <c r="G15" t="n">
-        <v>1.184356770833333</v>
+        <v>1.074109767469357</v>
       </c>
       <c r="H15" t="n">
-        <v>2.679818204781265</v>
+        <v>2.239009909050603</v>
       </c>
     </row>
     <row r="16">
@@ -1782,20 +1782,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.7684897835723414</v>
+        <v>0.8370011472178656</v>
       </c>
       <c r="F18" t="n">
-        <v>7.120289380208334</v>
+        <v>5.013165372826788</v>
       </c>
       <c r="G18" t="n">
-        <v>1.178119791666667</v>
+        <v>1.074109767469357</v>
       </c>
       <c r="H18" t="n">
-        <v>2.668387037183387</v>
+        <v>2.239009909050603</v>
       </c>
     </row>
     <row r="19">
@@ -1888,16 +1888,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.7689197068574851</v>
+        <v>0.836660225104804</v>
       </c>
       <c r="F21" t="n">
-        <v>7.107066731770833</v>
+        <v>5.023650716145833</v>
       </c>
       <c r="G21" t="n">
-        <v>1.187213541666667</v>
+        <v>1.09015625</v>
       </c>
       <c r="H21" t="n">
-        <v>2.665908237687643</v>
+        <v>2.241350199354361</v>
       </c>
     </row>
     <row r="22">
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.7708161427715885</v>
+        <v>0.8348522058453867</v>
       </c>
       <c r="F24" t="n">
-        <v>7.048740266927084</v>
+        <v>5.079257853190104</v>
       </c>
       <c r="G24" t="n">
-        <v>1.1812890625</v>
+        <v>1.096100260416667</v>
       </c>
       <c r="H24" t="n">
-        <v>2.654946377410867</v>
+        <v>2.253720890702774</v>
       </c>
     </row>
     <row r="25">
@@ -2099,16 +2099,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14.60794876394004</v>
+        <v>13.91403651561131</v>
       </c>
       <c r="C2" t="n">
-        <v>3.82203463667456</v>
+        <v>3.730152344826055</v>
       </c>
       <c r="D2" t="n">
-        <v>2.450784007202378</v>
+        <v>2.445973981812569</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5250348406759622</v>
+        <v>0.5475968134012457</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2133,16 +2133,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.384395011718749</v>
+        <v>5.065754947916666</v>
       </c>
       <c r="C3" t="n">
-        <v>2.717424334129425</v>
+        <v>2.250723205531206</v>
       </c>
       <c r="D3" t="n">
-        <v>1.2092265625</v>
+        <v>1.091197916666667</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7599026112474786</v>
+        <v>0.8352912414456735</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2167,16 +2167,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.277236195052044</v>
+        <v>5.896989963831719</v>
       </c>
       <c r="C4" t="n">
-        <v>2.697635296894679</v>
+        <v>2.42837187511133</v>
       </c>
       <c r="D4" t="n">
-        <v>1.226473334554635</v>
+        <v>1.169644306329891</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7633867899815057</v>
+        <v>0.8082643345096086</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2201,16 +2201,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.897482110004605</v>
+        <v>5.56198505153198</v>
       </c>
       <c r="C5" t="n">
-        <v>3.14602640008068</v>
+        <v>2.358386111630574</v>
       </c>
       <c r="D5" t="n">
-        <v>1.356159440869457</v>
+        <v>1.187743622503149</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6781916993787966</v>
+        <v>0.8191567372771731</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2235,16 +2235,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8.755208333333334</v>
+        <v>9.475260416666666</v>
       </c>
       <c r="C6" t="n">
-        <v>2.958920129596832</v>
+        <v>3.078191094891067</v>
       </c>
       <c r="D6" t="n">
-        <v>1.375</v>
+        <v>1.4765625</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7153317698360269</v>
+        <v>0.6919198823760808</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2609,16 +2609,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13.48114083660913</v>
+        <v>12.74180102904483</v>
       </c>
       <c r="C17" t="n">
-        <v>3.671667310175192</v>
+        <v>3.569565944067266</v>
       </c>
       <c r="D17" t="n">
-        <v>2.327680511277916</v>
+        <v>2.330081840530846</v>
       </c>
       <c r="E17" t="n">
-        <v>0.5616720520586753</v>
+        <v>0.5857110636385369</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2643,16 +2643,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7.315750317708333</v>
+        <v>5.091622989908855</v>
       </c>
       <c r="C18" t="n">
-        <v>2.704764373787176</v>
+        <v>2.256462494682518</v>
       </c>
       <c r="D18" t="n">
-        <v>1.209526041666667</v>
+        <v>1.09474609375</v>
       </c>
       <c r="E18" t="n">
-        <v>0.7621345356986301</v>
+        <v>0.8344501638320561</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2677,16 +2677,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>7.277808114731106</v>
+        <v>5.853000057075814</v>
       </c>
       <c r="C19" t="n">
-        <v>2.697741298703622</v>
+        <v>2.419297430469394</v>
       </c>
       <c r="D19" t="n">
-        <v>1.227003489121217</v>
+        <v>1.169847477459873</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7633681944944954</v>
+        <v>0.8096946293038061</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2711,16 +2711,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9.897482110004605</v>
+        <v>5.56198505153198</v>
       </c>
       <c r="C20" t="n">
-        <v>3.14602640008068</v>
+        <v>2.358386111630574</v>
       </c>
       <c r="D20" t="n">
-        <v>1.356159440869457</v>
+        <v>1.187743622503149</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6781916993787966</v>
+        <v>0.8191567372771731</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -2745,16 +2745,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9.12890625</v>
+        <v>9.440104166666666</v>
       </c>
       <c r="C21" t="n">
-        <v>3.021407991317955</v>
+        <v>3.072475250781797</v>
       </c>
       <c r="D21" t="n">
-        <v>1.388020833333333</v>
+        <v>1.46875</v>
       </c>
       <c r="E21" t="n">
-        <v>0.7031812965973205</v>
+        <v>0.6930629582556802</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -3119,16 +3119,16 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>14.62754429687408</v>
+        <v>13.9330943842419</v>
       </c>
       <c r="C32" t="n">
-        <v>3.824597272507797</v>
+        <v>3.732706040427226</v>
       </c>
       <c r="D32" t="n">
-        <v>2.449263688889946</v>
+        <v>2.443907239918674</v>
       </c>
       <c r="E32" t="n">
-        <v>0.5243977084151321</v>
+        <v>0.5469771628427191</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>7.181425610677084</v>
+        <v>5.125802473958334</v>
       </c>
       <c r="C33" t="n">
-        <v>2.679818204781265</v>
+        <v>2.264023514444657</v>
       </c>
       <c r="D33" t="n">
-        <v>1.184356770833333</v>
+        <v>1.093880208333333</v>
       </c>
       <c r="E33" t="n">
-        <v>0.7665019904937718</v>
+        <v>0.8333388466752456</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -3187,16 +3187,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>7.338588243826723</v>
+        <v>5.782931778991105</v>
       </c>
       <c r="C34" t="n">
-        <v>2.708982879943453</v>
+        <v>2.404772708384538</v>
       </c>
       <c r="D34" t="n">
-        <v>1.242082918155629</v>
+        <v>1.184504384191723</v>
       </c>
       <c r="E34" t="n">
-        <v>0.7613919797523615</v>
+        <v>0.8119728403929781</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -3221,16 +3221,16 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>9.04606133796708</v>
+        <v>5.013165372826788</v>
       </c>
       <c r="C35" t="n">
-        <v>3.007667092277182</v>
+        <v>2.239009909050603</v>
       </c>
       <c r="D35" t="n">
-        <v>1.33464218857777</v>
+        <v>1.074109767469357</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7058749291859038</v>
+        <v>0.8370011472178656</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>9.416666666666666</v>
+        <v>9.868489583333334</v>
       </c>
       <c r="C36" t="n">
-        <v>3.068658773253661</v>
+        <v>3.141415219822641</v>
       </c>
       <c r="D36" t="n">
-        <v>1.432291666666667</v>
+        <v>1.4609375</v>
       </c>
       <c r="E36" t="n">
-        <v>0.69382500884208</v>
+        <v>0.6791343669820415</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -3629,16 +3629,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>13.50822095005087</v>
+        <v>12.7674922675529</v>
       </c>
       <c r="C47" t="n">
-        <v>3.675353173512836</v>
+        <v>3.573162782123549</v>
       </c>
       <c r="D47" t="n">
-        <v>2.327165953683237</v>
+        <v>2.329059453452995</v>
       </c>
       <c r="E47" t="n">
-        <v>0.5607915649620119</v>
+        <v>0.5848757346413995</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3663,16 +3663,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.120289380208334</v>
+        <v>5.148455281575521</v>
       </c>
       <c r="C48" t="n">
-        <v>2.668387037183387</v>
+        <v>2.26902077592417</v>
       </c>
       <c r="D48" t="n">
-        <v>1.178119791666667</v>
+        <v>1.095162760416666</v>
       </c>
       <c r="E48" t="n">
-        <v>0.7684897835723414</v>
+        <v>0.8326023097012392</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3697,16 +3697,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>7.338588243826723</v>
+        <v>5.735743997122751</v>
       </c>
       <c r="C49" t="n">
-        <v>2.708982879943453</v>
+        <v>2.394941334797734</v>
       </c>
       <c r="D49" t="n">
-        <v>1.242082918155629</v>
+        <v>1.206632241081802</v>
       </c>
       <c r="E49" t="n">
-        <v>0.7613919797523615</v>
+        <v>0.8135071114049751</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3731,16 +3731,16 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>9.04606133796708</v>
+        <v>5.013165372826788</v>
       </c>
       <c r="C50" t="n">
-        <v>3.007667092277182</v>
+        <v>2.239009909050603</v>
       </c>
       <c r="D50" t="n">
-        <v>1.33464218857777</v>
+        <v>1.074109767469357</v>
       </c>
       <c r="E50" t="n">
-        <v>0.7058749291859038</v>
+        <v>0.8370011472178656</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3765,16 +3765,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>9.352864583333334</v>
+        <v>9.80859375</v>
       </c>
       <c r="C51" t="n">
-        <v>3.058245343875035</v>
+        <v>3.131867454091887</v>
       </c>
       <c r="D51" t="n">
-        <v>1.4140625</v>
+        <v>1.440104166666667</v>
       </c>
       <c r="E51" t="n">
-        <v>0.6958994798828346</v>
+        <v>0.6810818295917296</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -4139,16 +4139,16 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>14.66075845287511</v>
+        <v>13.97049005525031</v>
       </c>
       <c r="C62" t="n">
-        <v>3.828936987321039</v>
+        <v>3.737711874295598</v>
       </c>
       <c r="D62" t="n">
-        <v>2.453247114415234</v>
+        <v>2.445259063909666</v>
       </c>
       <c r="E62" t="n">
-        <v>0.5233177780873517</v>
+        <v>0.5457612740738328</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -4173,16 +4173,16 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>7.107066731770833</v>
+        <v>5.023650716145833</v>
       </c>
       <c r="C63" t="n">
-        <v>2.665908237687643</v>
+        <v>2.241350199354361</v>
       </c>
       <c r="D63" t="n">
-        <v>1.187213541666667</v>
+        <v>1.09015625</v>
       </c>
       <c r="E63" t="n">
-        <v>0.7689197068574851</v>
+        <v>0.836660225104804</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -4207,16 +4207,16 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>7.64877452991</v>
+        <v>5.685269249311088</v>
       </c>
       <c r="C64" t="n">
-        <v>2.765641793492064</v>
+        <v>2.384380265249461</v>
       </c>
       <c r="D64" t="n">
-        <v>1.287068127821274</v>
+        <v>1.201513333607042</v>
       </c>
       <c r="E64" t="n">
-        <v>0.7513065337277043</v>
+        <v>0.8151482553481539</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -4241,16 +4241,16 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>9.159287975851562</v>
+        <v>5.263494097740407</v>
       </c>
       <c r="C65" t="n">
-        <v>3.026431558098012</v>
+        <v>2.294230611281352</v>
       </c>
       <c r="D65" t="n">
-        <v>1.323886393965703</v>
+        <v>1.149518503727298</v>
       </c>
       <c r="E65" t="n">
-        <v>0.7021934603519439</v>
+        <v>0.8288619194157062</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -4275,16 +4275,16 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>9.143229166666666</v>
+        <v>8.180989583333334</v>
       </c>
       <c r="C66" t="n">
-        <v>3.023777301103153</v>
+        <v>2.860242923832403</v>
       </c>
       <c r="D66" t="n">
-        <v>1.380208333333333</v>
+        <v>1.393229166666667</v>
       </c>
       <c r="E66" t="n">
-        <v>0.7027155990167431</v>
+        <v>0.7340020092028192</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -4649,16 +4649,16 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>13.54405338304514</v>
+        <v>12.79610124920624</v>
       </c>
       <c r="C77" t="n">
-        <v>3.680224637579226</v>
+        <v>3.577163855515461</v>
       </c>
       <c r="D77" t="n">
-        <v>2.329489702574353</v>
+        <v>2.330287914262844</v>
       </c>
       <c r="E77" t="n">
-        <v>0.5596265035614609</v>
+        <v>0.5839455376816032</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -4683,16 +4683,16 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>7.048740266927084</v>
+        <v>5.079257853190104</v>
       </c>
       <c r="C78" t="n">
-        <v>2.654946377410867</v>
+        <v>2.253720890702774</v>
       </c>
       <c r="D78" t="n">
-        <v>1.1812890625</v>
+        <v>1.096100260416667</v>
       </c>
       <c r="E78" t="n">
-        <v>0.7708161427715885</v>
+        <v>0.8348522058453867</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -4717,16 +4717,16 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>7.64877452991</v>
+        <v>5.756730743914223</v>
       </c>
       <c r="C79" t="n">
-        <v>2.765641793492064</v>
+        <v>2.399318808310855</v>
       </c>
       <c r="D79" t="n">
-        <v>1.287068127821274</v>
+        <v>1.220251109563332</v>
       </c>
       <c r="E79" t="n">
-        <v>0.7513065337277043</v>
+        <v>0.8128247449964817</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4751,16 +4751,16 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>9.159287975851562</v>
+        <v>5.263494097740407</v>
       </c>
       <c r="C80" t="n">
-        <v>3.026431558098012</v>
+        <v>2.294230611281352</v>
       </c>
       <c r="D80" t="n">
-        <v>1.323886393965703</v>
+        <v>1.149518503727298</v>
       </c>
       <c r="E80" t="n">
-        <v>0.7021934603519439</v>
+        <v>0.8288619194157062</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -4785,16 +4785,16 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>9.220052083333334</v>
+        <v>8.092447916666666</v>
       </c>
       <c r="C81" t="n">
-        <v>3.036453866491855</v>
+        <v>2.844722818952079</v>
       </c>
       <c r="D81" t="n">
-        <v>1.393229166666667</v>
+        <v>1.372395833333333</v>
       </c>
       <c r="E81" t="n">
-        <v>0.7002177665390996</v>
+        <v>0.7368808669736625</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -5159,16 +5159,16 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>14.94827431030217</v>
+        <v>13.76629646971218</v>
       </c>
       <c r="C92" t="n">
-        <v>3.866299821573874</v>
+        <v>3.71029600836809</v>
       </c>
       <c r="D92" t="n">
-        <v>2.495309613221678</v>
+        <v>2.439560340245118</v>
       </c>
       <c r="E92" t="n">
-        <v>0.5341256147346998</v>
+        <v>0.5524004566486973</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5193,16 +5193,16 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>7.708303367904539</v>
+        <v>5.115532430013021</v>
       </c>
       <c r="C93" t="n">
-        <v>2.776383145011606</v>
+        <v>2.261754281528615</v>
       </c>
       <c r="D93" t="n">
-        <v>1.224106167056987</v>
+        <v>1.10529296875</v>
       </c>
       <c r="E93" t="n">
-        <v>0.7597648385080793</v>
+        <v>0.8336727685103763</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5227,16 +5227,16 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>7.678242188228045</v>
+        <v>6.176123219613963</v>
       </c>
       <c r="C94" t="n">
-        <v>2.770964126117125</v>
+        <v>2.485180721721051</v>
       </c>
       <c r="D94" t="n">
-        <v>1.28388548304942</v>
+        <v>1.237245725325212</v>
       </c>
       <c r="E94" t="n">
-        <v>0.7607017181311997</v>
+        <v>0.7991885516295013</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5261,16 +5261,16 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>10.24551051609158</v>
+        <v>6.019129328030568</v>
       </c>
       <c r="C95" t="n">
-        <v>3.200860902334181</v>
+        <v>2.453391393159797</v>
       </c>
       <c r="D95" t="n">
-        <v>1.373448728780005</v>
+        <v>1.160203012828579</v>
       </c>
       <c r="E95" t="n">
-        <v>0.6806908400039355</v>
+        <v>0.8042930758809059</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5295,16 +5295,16 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>9.254098360655737</v>
+        <v>7.203125</v>
       </c>
       <c r="C96" t="n">
-        <v>3.042054956876311</v>
+        <v>2.683863819197986</v>
       </c>
       <c r="D96" t="n">
-        <v>1.502732240437158</v>
+        <v>1.380208333333333</v>
       </c>
       <c r="E96" t="n">
-        <v>0.7115889569952663</v>
+        <v>0.7657964531131618</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5329,16 +5329,16 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>14.3507287695129</v>
+        <v>13.87265249496716</v>
       </c>
       <c r="C97" t="n">
-        <v>3.788235574711913</v>
+        <v>3.724600984664955</v>
       </c>
       <c r="D97" t="n">
-        <v>2.471510011728463</v>
+        <v>2.420509662653716</v>
       </c>
       <c r="E97" t="n">
-        <v>0.5527485778744226</v>
+        <v>0.5489423800017558</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5363,16 +5363,16 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>6.666466564207651</v>
+        <v>6.562653548177084</v>
       </c>
       <c r="C98" t="n">
-        <v>2.58195014750627</v>
+        <v>2.56176766085004</v>
       </c>
       <c r="D98" t="n">
-        <v>1.15957650273224</v>
+        <v>1.1729296875</v>
       </c>
       <c r="E98" t="n">
-        <v>0.792234478173077</v>
+        <v>0.7866208433183421</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -5397,16 +5397,16 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>8.287833824785851</v>
+        <v>8.009253332519807</v>
       </c>
       <c r="C99" t="n">
-        <v>2.878859813326424</v>
+        <v>2.830062425551742</v>
       </c>
       <c r="D99" t="n">
-        <v>1.329805644994232</v>
+        <v>1.323560415327578</v>
       </c>
       <c r="E99" t="n">
-        <v>0.7417033292169348</v>
+        <v>0.7395858688567298</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5431,16 +5431,16 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>7.38855596434879</v>
+        <v>7.327002620779894</v>
       </c>
       <c r="C100" t="n">
-        <v>2.718189832287067</v>
+        <v>2.706843663897103</v>
       </c>
       <c r="D100" t="n">
-        <v>1.276165604423903</v>
+        <v>1.300399789427047</v>
       </c>
       <c r="E100" t="n">
-        <v>0.7697300105392781</v>
+        <v>0.7617686765347249</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5465,16 +5465,16 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>6.953551912568306</v>
+        <v>7.127604166666667</v>
       </c>
       <c r="C101" t="n">
-        <v>2.636958837860065</v>
+        <v>2.669757323553335</v>
       </c>
       <c r="D101" t="n">
-        <v>1.207650273224044</v>
+        <v>1.265625</v>
       </c>
       <c r="E101" t="n">
-        <v>0.7832872440368919</v>
+        <v>0.7682519494471164</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5499,16 +5499,16 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>14.55867869860561</v>
+        <v>14.05633128457117</v>
       </c>
       <c r="C102" t="n">
-        <v>3.815583664212542</v>
+        <v>3.749177414389878</v>
       </c>
       <c r="D102" t="n">
-        <v>2.514117722757477</v>
+        <v>2.461773244413503</v>
       </c>
       <c r="E102" t="n">
-        <v>0.5462676595174947</v>
+        <v>0.5429702187504737</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -5533,16 +5533,16 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>4.891569721311476</v>
+        <v>4.812175697916667</v>
       </c>
       <c r="C103" t="n">
-        <v>2.211689336527957</v>
+        <v>2.193667180298021</v>
       </c>
       <c r="D103" t="n">
-        <v>1.115863387978142</v>
+        <v>1.12228125</v>
       </c>
       <c r="E103" t="n">
-        <v>0.8475504938166822</v>
+        <v>0.843536157335222</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -5567,16 +5567,16 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>7.111226623936073</v>
+        <v>6.947593417890073</v>
       </c>
       <c r="C104" t="n">
-        <v>2.666688325233392</v>
+        <v>2.635828791460112</v>
       </c>
       <c r="D104" t="n">
-        <v>1.337683242048498</v>
+        <v>1.337667319797364</v>
       </c>
       <c r="E104" t="n">
-        <v>0.7783731912368494</v>
+        <v>0.7741048474380903</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -5601,16 +5601,16 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>4.124780603089613</v>
+        <v>4.108910975744135</v>
       </c>
       <c r="C105" t="n">
-        <v>2.030955588655157</v>
+        <v>2.027044887451715</v>
       </c>
       <c r="D105" t="n">
-        <v>1.081322766388076</v>
+        <v>1.081957858672392</v>
       </c>
       <c r="E105" t="n">
-        <v>0.8714480623028008</v>
+        <v>0.8664022178760558</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5635,16 +5635,16 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>7.853825136612022</v>
+        <v>7.875</v>
       </c>
       <c r="C106" t="n">
-        <v>2.802467686988027</v>
+        <v>2.806243040080456</v>
       </c>
       <c r="D106" t="n">
-        <v>1.37431693989071</v>
+        <v>1.369791666666667</v>
       </c>
       <c r="E106" t="n">
-        <v>0.7552295414475622</v>
+        <v>0.7439510029697041</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5669,16 +5669,16 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>13.73486255045933</v>
+        <v>12.53775242113775</v>
       </c>
       <c r="C107" t="n">
-        <v>3.706057548185042</v>
+        <v>3.540868879404849</v>
       </c>
       <c r="D107" t="n">
-        <v>2.359791975084253</v>
+        <v>2.317662342011924</v>
       </c>
       <c r="E107" t="n">
-        <v>0.5719425189442293</v>
+        <v>0.5923455323877479</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5703,16 +5703,16 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>7.684071537303446</v>
+        <v>5.12874961751302</v>
       </c>
       <c r="C108" t="n">
-        <v>2.77201578951193</v>
+        <v>2.264674285082299</v>
       </c>
       <c r="D108" t="n">
-        <v>1.221291959406714</v>
+        <v>1.104407552083333</v>
       </c>
       <c r="E108" t="n">
-        <v>0.7605200420152398</v>
+        <v>0.8332430227830193</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -5737,16 +5737,16 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>7.681398184523484</v>
+        <v>6.143960426417496</v>
       </c>
       <c r="C109" t="n">
-        <v>2.771533543820728</v>
+        <v>2.478701358860622</v>
       </c>
       <c r="D109" t="n">
-        <v>1.286100831315334</v>
+        <v>1.239600762762587</v>
       </c>
       <c r="E109" t="n">
-        <v>0.7606033590963361</v>
+        <v>0.8002342977805678</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -5771,16 +5771,16 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>10.24551051609158</v>
+        <v>6.019129328030568</v>
       </c>
       <c r="C110" t="n">
-        <v>3.200860902334181</v>
+        <v>2.453391393159797</v>
       </c>
       <c r="D110" t="n">
-        <v>1.373448728780005</v>
+        <v>1.160203012828579</v>
       </c>
       <c r="E110" t="n">
-        <v>0.6806908400039355</v>
+        <v>0.8042930758809059</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -5805,16 +5805,16 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>9.209016393442623</v>
+        <v>7.203125</v>
       </c>
       <c r="C111" t="n">
-        <v>3.034636122081628</v>
+        <v>2.683863819197986</v>
       </c>
       <c r="D111" t="n">
-        <v>1.494535519125683</v>
+        <v>1.380208333333333</v>
       </c>
       <c r="E111" t="n">
-        <v>0.7129939709337305</v>
+        <v>0.7657964531131618</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -5839,16 +5839,16 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>12.71181801929431</v>
+        <v>12.31517698817004</v>
       </c>
       <c r="C112" t="n">
-        <v>3.565363658772315</v>
+        <v>3.509298646192718</v>
       </c>
       <c r="D112" t="n">
-        <v>2.307818342830007</v>
+        <v>2.262989260909706</v>
       </c>
       <c r="E112" t="n">
-        <v>0.6038264830836254</v>
+        <v>0.5995823852607594</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -5873,16 +5873,16 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>6.752357957650273</v>
+        <v>6.646635319010417</v>
       </c>
       <c r="C113" t="n">
-        <v>2.598529960891402</v>
+        <v>2.578106925441693</v>
       </c>
       <c r="D113" t="n">
-        <v>1.163811475409836</v>
+        <v>1.177513020833333</v>
       </c>
       <c r="E113" t="n">
-        <v>0.7895576072989532</v>
+        <v>0.7838902467226974</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -5907,16 +5907,16 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>8.288956617139855</v>
+        <v>8.010323493982217</v>
       </c>
       <c r="C114" t="n">
-        <v>2.879054813153069</v>
+        <v>2.830251489529193</v>
       </c>
       <c r="D114" t="n">
-        <v>1.330596416089928</v>
+        <v>1.324314119028163</v>
       </c>
       <c r="E114" t="n">
-        <v>0.7416683365357166</v>
+        <v>0.7395510734574777</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -5941,16 +5941,16 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>7.38855596434879</v>
+        <v>7.327002620779894</v>
       </c>
       <c r="C115" t="n">
-        <v>2.718189832287067</v>
+        <v>2.706843663897103</v>
       </c>
       <c r="D115" t="n">
-        <v>1.276165604423903</v>
+        <v>1.300399789427047</v>
       </c>
       <c r="E115" t="n">
-        <v>0.7697300105392781</v>
+        <v>0.7617686765347249</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -5975,16 +5975,16 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>6.8224043715847</v>
+        <v>7.002604166666667</v>
       </c>
       <c r="C116" t="n">
-        <v>2.611973271606105</v>
+        <v>2.646243406541935</v>
       </c>
       <c r="D116" t="n">
-        <v>1.19672131147541</v>
+        <v>1.255208333333333</v>
       </c>
       <c r="E116" t="n">
-        <v>0.787374557312424</v>
+        <v>0.772316219241248</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -6009,16 +6009,16 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>13.11534861965564</v>
+        <v>12.71046696320333</v>
       </c>
       <c r="C117" t="n">
-        <v>3.621511924549695</v>
+        <v>3.565174184132289</v>
       </c>
       <c r="D117" t="n">
-        <v>2.372963587099203</v>
+        <v>2.333089836208065</v>
       </c>
       <c r="E117" t="n">
-        <v>0.5912501437365807</v>
+        <v>0.5867298644171525</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -6043,16 +6043,16 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>4.908395950819672</v>
+        <v>4.827398354166667</v>
       </c>
       <c r="C118" t="n">
-        <v>2.215490002419255</v>
+        <v>2.197134122935299</v>
       </c>
       <c r="D118" t="n">
-        <v>1.120125683060109</v>
+        <v>1.126135416666667</v>
       </c>
       <c r="E118" t="n">
-        <v>0.8470260915234316</v>
+        <v>0.8430412054793553</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -6077,16 +6077,16 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>7.111226623936073</v>
+        <v>6.947593417890073</v>
       </c>
       <c r="C119" t="n">
-        <v>2.666688325233392</v>
+        <v>2.635828791460112</v>
       </c>
       <c r="D119" t="n">
-        <v>1.337683242048498</v>
+        <v>1.337667319797364</v>
       </c>
       <c r="E119" t="n">
-        <v>0.7783731912368494</v>
+        <v>0.7741048474380903</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -6111,16 +6111,16 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>4.124780603089613</v>
+        <v>4.108910975744135</v>
       </c>
       <c r="C120" t="n">
-        <v>2.030955588655157</v>
+        <v>2.027044887451715</v>
       </c>
       <c r="D120" t="n">
-        <v>1.081322766388076</v>
+        <v>1.081957858672392</v>
       </c>
       <c r="E120" t="n">
-        <v>0.8714480623028008</v>
+        <v>0.8664022178760558</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -6145,16 +6145,16 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>7.896174863387978</v>
+        <v>7.915364583333333</v>
       </c>
       <c r="C121" t="n">
-        <v>2.810013320855967</v>
+        <v>2.813425773560293</v>
       </c>
       <c r="D121" t="n">
-        <v>1.39344262295082</v>
+        <v>1.388020833333333</v>
       </c>
       <c r="E121" t="n">
-        <v>0.7539096798690049</v>
+        <v>0.742638582515349</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -6240,16 +6240,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7684014337337335</v>
+        <v>0.7625833435452005</v>
       </c>
       <c r="E2" t="n">
-        <v>7.431185332177795</v>
+        <v>7.301946858867508</v>
       </c>
       <c r="F2" t="n">
-        <v>1.461107580309341</v>
+        <v>1.453374252935564</v>
       </c>
       <c r="G2" t="n">
-        <v>2.668931832342693</v>
+        <v>2.647721551907941</v>
       </c>
     </row>
     <row r="3">
@@ -6313,36 +6313,36 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>drop</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>robust</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>zscore</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7597737896642778</v>
+        <v>0.759473054982568</v>
       </c>
       <c r="E5" t="n">
-        <v>7.70801615671096</v>
+        <v>7.397606372143528</v>
       </c>
       <c r="F5" t="n">
-        <v>1.484660811812581</v>
+        <v>1.433710724260695</v>
       </c>
       <c r="G5" t="n">
-        <v>2.705476920323415</v>
+        <v>2.673831396952504</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>drop</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6352,31 +6352,31 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>zscore</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.7588234559079498</v>
+        <v>0.7591824763890805</v>
       </c>
       <c r="E6" t="n">
-        <v>7.417585332311118</v>
+        <v>7.406543358619767</v>
       </c>
       <c r="F6" t="n">
-        <v>1.474271432047075</v>
+        <v>1.440416400603951</v>
       </c>
       <c r="G6" t="n">
-        <v>2.670403692621864</v>
+        <v>2.684299947141111</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>robust</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -6385,22 +6385,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7541928888739091</v>
+        <v>0.7588234559079498</v>
       </c>
       <c r="E7" t="n">
-        <v>7.56000227522441</v>
+        <v>7.417585332311118</v>
       </c>
       <c r="F7" t="n">
-        <v>1.474694267909985</v>
+        <v>1.474271432047075</v>
       </c>
       <c r="G7" t="n">
-        <v>2.682392262736036</v>
+        <v>2.670403692621864</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>median</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6414,22 +6414,22 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.752499335738111</v>
+        <v>0.7541928888739091</v>
       </c>
       <c r="E8" t="n">
-        <v>7.612088911372538</v>
+        <v>7.56000227522441</v>
       </c>
       <c r="F8" t="n">
-        <v>1.493318797654427</v>
+        <v>1.474694267909985</v>
       </c>
       <c r="G8" t="n">
-        <v>2.693331512129927</v>
+        <v>2.682392262736036</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>drop</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6443,196 +6443,196 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.7503464079802475</v>
+        <v>0.7541928888739091</v>
       </c>
       <c r="E9" t="n">
-        <v>7.678303996336015</v>
+        <v>7.56000227522441</v>
       </c>
       <c r="F9" t="n">
-        <v>1.496554686975512</v>
+        <v>1.474694267909985</v>
       </c>
       <c r="G9" t="n">
-        <v>2.7055008119037</v>
+        <v>2.682392262736036</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>drop</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>zscore</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.7384313989539995</v>
+        <v>0.752499335738111</v>
       </c>
       <c r="E10" t="n">
-        <v>8.392818586003585</v>
+        <v>7.612088911372538</v>
       </c>
       <c r="F10" t="n">
-        <v>1.455022630045817</v>
+        <v>1.493318797654427</v>
       </c>
       <c r="G10" t="n">
-        <v>2.874622307341991</v>
+        <v>2.693331512129927</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.7319436368633315</v>
+        <v>0.7520867366290632</v>
       </c>
       <c r="E11" t="n">
-        <v>8.244296537711081</v>
+        <v>7.624778740356194</v>
       </c>
       <c r="F11" t="n">
-        <v>1.462879937893037</v>
+        <v>1.455935263582135</v>
       </c>
       <c r="G11" t="n">
-        <v>2.8513450755519</v>
+        <v>2.703583174802635</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>drop</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.7318582799590385</v>
+        <v>0.7510702611565285</v>
       </c>
       <c r="E12" t="n">
-        <v>8.246921760340751</v>
+        <v>7.656041289473947</v>
       </c>
       <c r="F12" t="n">
-        <v>1.459459520639837</v>
+        <v>1.464502076096448</v>
       </c>
       <c r="G12" t="n">
-        <v>2.851317214600118</v>
+        <v>2.718897244795108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>zscore</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.7314217202433815</v>
+        <v>0.7503464079802475</v>
       </c>
       <c r="E13" t="n">
-        <v>8.260348517721848</v>
+        <v>7.678303996336015</v>
       </c>
       <c r="F13" t="n">
-        <v>1.464084904706317</v>
+        <v>1.496554686975512</v>
       </c>
       <c r="G13" t="n">
-        <v>2.854148826320528</v>
+        <v>2.7055008119037</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>drop</t>
+          <t>median</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>robust</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.7279407279681209</v>
+        <v>0.7498136265114418</v>
       </c>
       <c r="E14" t="n">
-        <v>8.7294274070847</v>
+        <v>7.694690133815593</v>
       </c>
       <c r="F14" t="n">
-        <v>1.488941607420576</v>
+        <v>1.429013677817497</v>
       </c>
       <c r="G14" t="n">
-        <v>2.920838841138348</v>
+        <v>2.721600451197589</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>robust</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.7214742162190524</v>
+        <v>0.7484151104614505</v>
       </c>
       <c r="E15" t="n">
-        <v>8.566292282783042</v>
+        <v>7.737702658845629</v>
       </c>
       <c r="F15" t="n">
-        <v>1.492709522129138</v>
+        <v>1.450233806848774</v>
       </c>
       <c r="G15" t="n">
-        <v>2.895841381991699</v>
+        <v>2.73523744632631</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>median</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6642,26 +6642,26 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.721360312483511</v>
+        <v>0.74168487282217</v>
       </c>
       <c r="E16" t="n">
-        <v>8.569795486965806</v>
+        <v>7.944696718670292</v>
       </c>
       <c r="F16" t="n">
-        <v>1.495804948216018</v>
+        <v>1.451467819982617</v>
       </c>
       <c r="G16" t="n">
-        <v>2.896906652148339</v>
+        <v>2.756385478425933</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6671,26 +6671,26 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>iqr</t>
+          <t>isolation_forest</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.7210339436317338</v>
+        <v>0.7404458018019563</v>
       </c>
       <c r="E17" t="n">
-        <v>8.579833232622121</v>
+        <v>7.982805379111669</v>
       </c>
       <c r="F17" t="n">
-        <v>1.496604910981668</v>
+        <v>1.474224465462455</v>
       </c>
       <c r="G17" t="n">
-        <v>2.898606411703435</v>
+        <v>2.769164926398047</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6700,26 +6700,26 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.6984895474710907</v>
+        <v>0.7319436368633315</v>
       </c>
       <c r="E18" t="n">
-        <v>9.273204899077268</v>
+        <v>8.244296537711081</v>
       </c>
       <c r="F18" t="n">
-        <v>1.499214670416661</v>
+        <v>1.462879937893037</v>
       </c>
       <c r="G18" t="n">
-        <v>3.023727105358379</v>
+        <v>2.8513450755519</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>drop</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6729,26 +6729,26 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.6973501461986943</v>
+        <v>0.7318582799590385</v>
       </c>
       <c r="E19" t="n">
-        <v>9.710971836364093</v>
+        <v>8.246921760340751</v>
       </c>
       <c r="F19" t="n">
-        <v>1.547033802742398</v>
+        <v>1.459459520639837</v>
       </c>
       <c r="G19" t="n">
-        <v>3.097020781186702</v>
+        <v>2.851317214600118</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>drop</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6758,26 +6758,26 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.6968320813903595</v>
+        <v>0.7314217202433815</v>
       </c>
       <c r="E20" t="n">
-        <v>9.324181647813425</v>
+        <v>8.260348517721848</v>
       </c>
       <c r="F20" t="n">
-        <v>1.502992490705599</v>
+        <v>1.464084904706317</v>
       </c>
       <c r="G20" t="n">
-        <v>3.032739646614405</v>
+        <v>2.854148826320528</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>median</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6787,26 +6787,26 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.6937095556455837</v>
+        <v>0.7314217202433815</v>
       </c>
       <c r="E21" t="n">
-        <v>9.420217525810633</v>
+        <v>8.260348517721848</v>
       </c>
       <c r="F21" t="n">
-        <v>1.501678063253718</v>
+        <v>1.464084904706317</v>
       </c>
       <c r="G21" t="n">
-        <v>3.048321474812925</v>
+        <v>2.854148826320528</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>median</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6816,26 +6816,26 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.6903983233378498</v>
+        <v>0.7214742162190524</v>
       </c>
       <c r="E22" t="n">
-        <v>9.522057231202329</v>
+        <v>8.566292282783042</v>
       </c>
       <c r="F22" t="n">
-        <v>1.528527446624669</v>
+        <v>1.492709522129138</v>
       </c>
       <c r="G22" t="n">
-        <v>3.057944844552671</v>
+        <v>2.895841381991699</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6845,20 +6845,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.6896906156082456</v>
+        <v>0.721360312483511</v>
       </c>
       <c r="E23" t="n">
-        <v>9.543823371414835</v>
+        <v>8.569795486965806</v>
       </c>
       <c r="F23" t="n">
-        <v>1.526324702240442</v>
+        <v>1.495804948216018</v>
       </c>
       <c r="G23" t="n">
-        <v>3.062139175540382</v>
+        <v>2.896906652148339</v>
       </c>
     </row>
     <row r="24">
@@ -6874,26 +6874,26 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.6893743936746362</v>
+        <v>0.7210339436317338</v>
       </c>
       <c r="E24" t="n">
-        <v>9.966885748636415</v>
+        <v>8.579833232622121</v>
       </c>
       <c r="F24" t="n">
-        <v>1.57589644650905</v>
+        <v>1.496604910981668</v>
       </c>
       <c r="G24" t="n">
-        <v>3.13131259038262</v>
+        <v>2.898606411703435</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>median</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6903,20 +6903,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>isolation_forest</t>
+          <t>iqr</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.688369542223954</v>
+        <v>0.7210339436317338</v>
       </c>
       <c r="E25" t="n">
-        <v>9.584454082809753</v>
+        <v>8.579833232622121</v>
       </c>
       <c r="F25" t="n">
-        <v>1.523528669025294</v>
+        <v>1.496604910981668</v>
       </c>
       <c r="G25" t="n">
-        <v>3.068408159475235</v>
+        <v>2.898606411703435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>